<commit_message>
D35: the app grows two faces, and the back office gets a front door
The founder looked at a nine-entry rail heading for twelve and asked
for his portal's card layout. Half yes: a card hub is exactly right for
the surfaces a manager visits (Menu, Reports, Settings, and everything
still coming: inventory, guests, food cost), and exactly wrong in front
of the screen a server taps two hundred times a shift. So the floor
keeps the rail and the management surfaces collapse into one Office
entry opening a card hub, each card carrying a live one-line stat and
obeying the same role matrix as everything else: absent, never grayed.
Sign-in lands by role: servers on Service, kitchen on the KDS, managers
and the owner on the hub. Incumbents split POS from back office for the
same reason.

Ticket UI-T5, batched into the E25-T2 session after the roles engine
merges. Tracking log refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ticket_Tracking_Log.xlsx
+++ b/Ticket_Tracking_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/005_POS System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AE9D50C-18FA-4435-854B-0CCC7427194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9AD110B8-5DB9-468A-8879-488821EF5839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE14EA74-6406-48C7-8E94-002559044C9F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AF7D2503-88DE-4FD1-841B-144F9D868AA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="How to use" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tickets!$A$1:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tickets!$A$1:$G$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="193">
   <si>
     <t>Ticket</t>
   </si>
@@ -469,10 +469,25 @@
     <t>Every page's rail obeys the signed-in role; calm refusal page</t>
   </si>
   <si>
-    <t>Ready (after E25-T1)</t>
+    <t>Ready (after E25-T1; batch with UI-T5)</t>
   </si>
   <si>
     <t>docs/tickets/E25-T2-roles-ui.md</t>
+  </si>
+  <si>
+    <t>UI-T5</t>
+  </si>
+  <si>
+    <t>App shell (D35)</t>
+  </si>
+  <si>
+    <t>Back-office card hub at /office; floor keeps the rail; land by role</t>
+  </si>
+  <si>
+    <t>Ready (after E25-T2; batch with E25-T2)</t>
+  </si>
+  <si>
+    <t>docs/tickets/UI-T5-back-office-hub.md</t>
   </si>
   <si>
     <t>E26-T2</t>
@@ -1045,8 +1060,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDDE5EF9-DE2A-42B6-92BD-D4CCA740038B}">
-  <dimension ref="A1:G42"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AEE10CC-4F8B-4BF5-B542-FCA411AA1589}">
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1975,55 +1990,76 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="C41" s="10" t="s">
+      <c r="B41" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D41" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" s="5" t="s">
+      <c r="C41" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5" t="s">
+      <c r="D41" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E41" s="4" t="s">
         <v>146</v>
+      </c>
+      <c r="F41" s="4"/>
+      <c r="G41" s="4" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>131</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>107</v>
+        <v>10</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F42" s="5"/>
       <c r="G42" s="5" t="s">
-        <v>146</v>
+        <v>151</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E43" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G42" xr:uid="{FDDE5EF9-DE2A-42B6-92BD-D4CCA740038B}"/>
+  <autoFilter ref="A1:G43" xr:uid="{6AEE10CC-4F8B-4BF5-B542-FCA411AA1589}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01C69DD-7655-459E-AA8B-066CF3F11028}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82FCF77C-8ABF-42A1-A2EE-26D6371DC281}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2034,134 +2070,134 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="B6" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C6" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C7" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B8" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C8" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B9" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C9" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C10" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B11" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C11" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C12" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2170,7 +2206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E26D3E84-1BC8-42BE-A287-D55B5CFA17CF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B74B1218-1541-45B3-9305-4A1285002D26}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2179,32 +2215,32 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
E25-T3 ticketed: the chef could not leave
Founder-reported the day after the roles wave merged: Nico cannot sign
out, because the terminal sheet lives only on Service and the roles
wave correctly made Service unreachable for a kitchen sign-in. The one
Sign out a kitchen user can reach is on the trespass-refusal page,
which only appears by going somewhere they should not. The fix ticket
puts the identity chip and the terminal sheet on every page, KDS night
theme included. Tracking log refreshed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ticket_Tracking_Log.xlsx
+++ b/Ticket_Tracking_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/005_POS System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA08B1E9-DE50-4EF3-973C-75C8D84B98E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{387B01C8-5D47-4690-9AEF-FAEC7ABDAC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6959A93D-758A-41C3-A9D6-39AA66465C52}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6AEE6259-8A6F-40FC-B149-377D5CB212DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="How to use" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tickets!$A$1:$G$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tickets!$A$1:$G$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="194">
   <si>
     <t>Ticket</t>
   </si>
@@ -479,6 +479,18 @@
   </si>
   <si>
     <t>docs/tickets/UI-T5-back-office-hub.md</t>
+  </si>
+  <si>
+    <t>E25-T3</t>
+  </si>
+  <si>
+    <t>Terminal sheet (sign in / out / clock out) on every page; kitchen can finally sign out</t>
+  </si>
+  <si>
+    <t>READY TO FIRE</t>
+  </si>
+  <si>
+    <t>docs/tickets/E25-T3-terminal-sheet-everywhere.md</t>
   </si>
   <si>
     <t>E26-T2</t>
@@ -653,7 +665,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -663,6 +675,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDAEFE2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB4E0C6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -691,14 +709,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1035,8 +1055,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F387A276-AFF0-42DF-98AA-FA0A7A5663B2}">
-  <dimension ref="A1:G43"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE2FC319-973E-4F77-935B-0B41D2CC0871}">
+  <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1049,25 +1069,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1078,7 +1098,7 @@
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -1101,7 +1121,7 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1124,7 +1144,7 @@
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1147,7 +1167,7 @@
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1170,7 +1190,7 @@
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -1193,7 +1213,7 @@
       <c r="B7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -1216,7 +1236,7 @@
       <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1239,7 +1259,7 @@
       <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -1262,7 +1282,7 @@
       <c r="B10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>38</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1285,7 +1305,7 @@
       <c r="B11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -1308,7 +1328,7 @@
       <c r="B12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1331,7 +1351,7 @@
       <c r="B13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>47</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1354,7 +1374,7 @@
       <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>51</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1377,7 +1397,7 @@
       <c r="B15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>54</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1400,7 +1420,7 @@
       <c r="B16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>58</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -1423,7 +1443,7 @@
       <c r="B17" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>61</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1446,7 +1466,7 @@
       <c r="B18" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>64</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -1469,7 +1489,7 @@
       <c r="B19" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -1492,7 +1512,7 @@
       <c r="B20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>71</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1515,7 +1535,7 @@
       <c r="B21" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="6" t="s">
         <v>75</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -1538,7 +1558,7 @@
       <c r="B22" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>78</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1561,7 +1581,7 @@
       <c r="B23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>81</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1584,7 +1604,7 @@
       <c r="B24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>85</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1607,7 +1627,7 @@
       <c r="B25" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>89</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1630,7 +1650,7 @@
       <c r="B26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>93</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1653,7 +1673,7 @@
       <c r="B27" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>96</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -1676,7 +1696,7 @@
       <c r="B28" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>100</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1699,7 +1719,7 @@
       <c r="B29" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>103</v>
       </c>
       <c r="D29" s="1" t="s">
@@ -1722,7 +1742,7 @@
       <c r="B30" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="6" t="s">
         <v>106</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -1745,7 +1765,7 @@
       <c r="B31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="6" t="s">
         <v>110</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -1768,7 +1788,7 @@
       <c r="B32" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="6" t="s">
         <v>113</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1791,7 +1811,7 @@
       <c r="B33" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="6" t="s">
         <v>116</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1814,7 +1834,7 @@
       <c r="B34" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="6" t="s">
         <v>119</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -1837,7 +1857,7 @@
       <c r="B35" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="6" t="s">
         <v>122</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1860,7 +1880,7 @@
       <c r="B36" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="6" t="s">
         <v>125</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1883,7 +1903,7 @@
       <c r="B37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>128</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -1906,7 +1926,7 @@
       <c r="B38" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="6" t="s">
         <v>132</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -1929,7 +1949,7 @@
       <c r="B39" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>136</v>
       </c>
       <c r="D39" s="1" t="s">
@@ -1952,7 +1972,7 @@
       <c r="B40" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -1975,7 +1995,7 @@
       <c r="B41" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>143</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -1996,13 +2016,13 @@
         <v>145</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="C42" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C42" s="7" t="s">
         <v>146</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>147</v>
@@ -2013,34 +2033,55 @@
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
+      <c r="A43" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="B43" s="3" t="s">
+      <c r="B43" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="D43" s="3" t="s">
+      <c r="D43" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F43" s="4"/>
+      <c r="G43" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="D44" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F43" s="3"/>
-      <c r="G43" s="3" t="s">
-        <v>148</v>
+      <c r="E44" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="F44" s="4"/>
+      <c r="G44" s="4" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G43" xr:uid="{F387A276-AFF0-42DF-98AA-FA0A7A5663B2}"/>
+  <autoFilter ref="A1:G44" xr:uid="{CE2FC319-973E-4F77-935B-0B41D2CC0871}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9633AFA5-1EB6-409D-9F89-2D78B5FF707D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A366FFDB-3764-46F6-9498-BCAF89B014E0}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2050,135 +2091,135 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>153</v>
+      <c r="A1" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" t="s">
         <v>160</v>
-      </c>
-      <c r="C4" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B5" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B6" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C6" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B8" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B9" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C9" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B10" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C10" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B11" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C11" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B12" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C12" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2187,7 +2228,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{534B9455-27A9-4E63-B2EB-4FA9BC2E6280}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262959A8-C1B0-489B-B9C4-DDA6B694E459}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2195,33 +2236,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
-        <v>184</v>
+      <c r="A1" s="9" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>187</v>
+      <c r="A6" s="10" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="9" t="s">
-        <v>189</v>
+      <c r="A10" s="11" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Review pass: E25-T3 merges; the chef can go home
Verified with my own screenshots: the KDS topbar carries the Nico F.
Kitchen chip in the night tokens, tapping it opens the full terminal
sheet, and Sign out lands him on the lock screen he could not reach
yesterday. The self-contained sheet component and the mid-switch rerun
of each page's own visibility logic are the right shapes, and the
variable-shadowing catch was real.

One suite failure during review was the clock, not the code: the
E23-T2 book test books at now minus twenty minutes, so in the first
twenty minutes after midnight the row lands on yesterday's service
date. Third member of the midnight-flake family; the review ran at
00:11. Confirmed by diff that this ticket never touched the test;
flagged for the next engine ticket to fix by the established pattern.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ticket_Tracking_Log.xlsx
+++ b/Ticket_Tracking_Log.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0b0a87718b906f2e/005_POS System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{387B01C8-5D47-4690-9AEF-FAEC7ABDAC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2993CF28-332A-495B-B982-115EEAB2F743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6AEE6259-8A6F-40FC-B149-377D5CB212DC}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D745ECD8-F88A-44C7-8644-B915AD88A243}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="193">
   <si>
     <t>Ticket</t>
   </si>
@@ -485,9 +485,6 @@
   </si>
   <si>
     <t>Terminal sheet (sign in / out / clock out) on every page; kitchen can finally sign out</t>
-  </si>
-  <si>
-    <t>READY TO FIRE</t>
   </si>
   <si>
     <t>docs/tickets/E25-T3-terminal-sheet-everywhere.md</t>
@@ -665,7 +662,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -675,12 +672,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDAEFE2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB4E0C6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -709,16 +700,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -1055,7 +1044,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE2FC319-973E-4F77-935B-0B41D2CC0871}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2B4FE54-4911-4935-B1B2-3C87EBCD39BA}">
   <dimension ref="A1:G44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1069,25 +1058,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="5" t="s">
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1098,7 +1087,7 @@
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -1121,7 +1110,7 @@
       <c r="B3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1144,7 +1133,7 @@
       <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1167,7 +1156,7 @@
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1190,7 +1179,7 @@
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="5" t="s">
         <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -1213,7 +1202,7 @@
       <c r="B7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -1236,7 +1225,7 @@
       <c r="B8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1259,7 +1248,7 @@
       <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="5" t="s">
         <v>34</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -1282,7 +1271,7 @@
       <c r="B10" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1305,7 +1294,7 @@
       <c r="B11" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -1328,7 +1317,7 @@
       <c r="B12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1351,7 +1340,7 @@
       <c r="B13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1374,7 +1363,7 @@
       <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1397,7 +1386,7 @@
       <c r="B15" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>54</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1420,7 +1409,7 @@
       <c r="B16" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>58</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -1443,7 +1432,7 @@
       <c r="B17" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1466,7 +1455,7 @@
       <c r="B18" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>64</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -1489,7 +1478,7 @@
       <c r="B19" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="5" t="s">
         <v>67</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -1512,7 +1501,7 @@
       <c r="B20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1535,7 +1524,7 @@
       <c r="B21" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="5" t="s">
         <v>75</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -1558,7 +1547,7 @@
       <c r="B22" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="5" t="s">
         <v>78</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1581,7 +1570,7 @@
       <c r="B23" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>81</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1604,7 +1593,7 @@
       <c r="B24" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1627,7 +1616,7 @@
       <c r="B25" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="5" t="s">
         <v>89</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1650,7 +1639,7 @@
       <c r="B26" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="5" t="s">
         <v>93</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1673,7 +1662,7 @@
       <c r="B27" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="5" t="s">
         <v>96</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -1696,7 +1685,7 @@
       <c r="B28" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>100</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1719,7 +1708,7 @@
       <c r="B29" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="5" t="s">
         <v>103</v>
       </c>
       <c r="D29" s="1" t="s">
@@ -1742,7 +1731,7 @@
       <c r="B30" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="5" t="s">
         <v>106</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -1765,7 +1754,7 @@
       <c r="B31" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="5" t="s">
         <v>110</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -1788,7 +1777,7 @@
       <c r="B32" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="5" t="s">
         <v>113</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1811,7 +1800,7 @@
       <c r="B33" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" s="5" t="s">
         <v>116</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1834,7 +1823,7 @@
       <c r="B34" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="5" t="s">
         <v>119</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -1857,7 +1846,7 @@
       <c r="B35" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" s="5" t="s">
         <v>122</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1880,7 +1869,7 @@
       <c r="B36" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="5" t="s">
         <v>125</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1903,7 +1892,7 @@
       <c r="B37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="5" t="s">
         <v>128</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -1926,7 +1915,7 @@
       <c r="B38" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" s="5" t="s">
         <v>132</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -1949,7 +1938,7 @@
       <c r="B39" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C39" s="6" t="s">
+      <c r="C39" s="5" t="s">
         <v>136</v>
       </c>
       <c r="D39" s="1" t="s">
@@ -1972,7 +1961,7 @@
       <c r="B40" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="C40" s="5" t="s">
         <v>139</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -1995,7 +1984,7 @@
       <c r="B41" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>143</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -2012,76 +2001,78 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
+      <c r="A42" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B42" s="3" t="s">
+      <c r="B42" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="C42" s="7" t="s">
+      <c r="C42" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D42" s="3" t="s">
+      <c r="D42" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E42" s="3" t="s">
+      <c r="E42" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F42" s="2">
+        <v>46270</v>
+      </c>
+      <c r="G42" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F42" s="3"/>
-      <c r="G42" s="3" t="s">
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
+      <c r="B43" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B43" s="4" t="s">
+      <c r="D43" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C44" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E44" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="D43" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" s="4" t="s">
+      <c r="F44" s="3"/>
+      <c r="G44" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F43" s="4"/>
-      <c r="G43" s="4" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="F44" s="4"/>
-      <c r="G44" s="4" t="s">
-        <v>152</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G44" xr:uid="{CE2FC319-973E-4F77-935B-0B41D2CC0871}"/>
+  <autoFilter ref="A1:G44" xr:uid="{C2B4FE54-4911-4935-B1B2-3C87EBCD39BA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A366FFDB-3764-46F6-9498-BCAF89B014E0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A131D7A1-BDA5-468C-A2EA-EF218F1BF5B1}">
   <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2091,135 +2082,135 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" t="s">
         <v>158</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>159</v>
-      </c>
-      <c r="C2" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B3" t="s">
         <v>161</v>
       </c>
-      <c r="B3" t="s">
-        <v>162</v>
-      </c>
       <c r="C3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" t="s">
         <v>163</v>
       </c>
-      <c r="B4" t="s">
-        <v>164</v>
-      </c>
       <c r="C4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>164</v>
+      </c>
+      <c r="B5" t="s">
         <v>165</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>166</v>
-      </c>
-      <c r="C5" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" t="s">
         <v>168</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>169</v>
-      </c>
-      <c r="C6" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B7" t="s">
         <v>171</v>
       </c>
-      <c r="B7" t="s">
-        <v>172</v>
-      </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>172</v>
+      </c>
+      <c r="B8" t="s">
         <v>173</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>174</v>
-      </c>
-      <c r="C8" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>175</v>
+      </c>
+      <c r="B9" t="s">
         <v>176</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>177</v>
-      </c>
-      <c r="C9" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>178</v>
+      </c>
+      <c r="B10" t="s">
         <v>179</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>180</v>
-      </c>
-      <c r="C10" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" t="s">
         <v>182</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>183</v>
-      </c>
-      <c r="C11" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>184</v>
+      </c>
+      <c r="B12" t="s">
         <v>185</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>186</v>
-      </c>
-      <c r="C12" t="s">
-        <v>187</v>
       </c>
     </row>
   </sheetData>
@@ -2228,7 +2219,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262959A8-C1B0-489B-B9C4-DDA6B694E459}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4C4CD3-92DA-4378-A802-033CE836374B}">
   <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2236,33 +2227,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>188</v>
+      <c r="A1" s="7" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>190</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>192</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>